<commit_message>
MTDF v1.1.6: claims-and-provenance audit + verification pass
Papers (HTML canonical; TeX regenerated from HTML; PDFs rebuilt): claims
re-graded without changing results; text-level number corrections restoring
agreement with pipeline artifacts (k_f transcription, S8 0.013 harmonisation,
z_t 0.74, 15/15 scalar pillars, gamma_low direction); E_G consistency test
rebuilt on six verified literature measurements with the z-dependent GR
baseline (previous +2.9 sigma tension was an artefact of a wrong constant);
synthesis figure relabelled as illustrative; MTDF_08 evidence grading with
the dated pre-registration record; verified reference entries added across
the suite; suite extent, dates and cross-document labels unified. Figures
regenerated from corrected scripts. Dashboard regenerated (cwd-independent
workbook lookup). Full details in CHANGELOG [v1.1.6].

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/validation/data/DB_Workbook_STRICT_V18.xlsx
+++ b/validation/data/DB_Workbook_STRICT_V18.xlsx
@@ -950,12 +950,12 @@
       <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Elastic-field cosmological framework treating spacetime as a deformable medium with stress tensor F_μν = E S̃_μν. 
-Parameters α, β, δ_bf, κ are empirical; E, τ, γ, β_eos are derived from first principles.</t>
+Parameter provenance: β is anchored to void statistics; α is a frozen, void-motivated coupling (not independently measured); δ_bf is fixed post hoc from cluster baryon fractions; κ is theory-motivated and FIRAS-bounded; E and γ are derived; τ is synchronised to the age of the universe; β_eos is a fitted phenomenological exponent.</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>Four fundamental parameters (α, β, τ, β_eos) with all remaining quantities derived or externally constrained. Reproduces major cosmic phenomena without dark matter or dark energy.</t>
+          <t>Four fundamental parameters (one anchored β, one frozen void-motivated α, one synchronised τ, one fitted β_eos), with remaining quantities derived or externally constrained. Reproduces a broad set of cosmic phenomena without separate dark components; the economy claim is zero per-observable tuning, not parameter-count reduction.</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
-          <t>Consistent if one fixed parameter set, derived entirely from empirical or first-principles data and with no fitted parameters,
+          <t>Consistent if one parameter set, fixed in advance with no per-pillar fitting,
 reproduces all pillars within observational bands.</t>
         </is>
       </c>
@@ -981,9 +981,9 @@
       </c>
       <c r="I3" s="11" t="inlineStr">
         <is>
-          <t>DOI: 10.1093/mnras/staa2785 (measurement of α)
+          <t>DOI: 10.1088/0004-637X/761/1/44 (Sutter et al. 2012 SDSS DR7 void catalog: void-dynamics data motivating α; α itself is frozen, not directly measured)
 DOI: 10.1088/0004-637X/761/1/44 (void quantization β: MTDF-original ansatz Rₙ = β(1+√n) matched to Sutter et al. 2012 SDSS DR7 void radii)
-DOI: 10.1051/0004-6361/201935943 (cluster baryon fraction δ_bf)
+DOI: 10.1088/0004-637X/703/1/982 and DOI: 10.1088/0004-637X/778/1/14 (Giodini et al. 2009; Gonzalez et al. 2013, cluster baryon fractions, δ_bf)
 DOI: 10.1103/PhysRevD.85.054503 (CMB polarization β_eos)</t>
         </is>
       </c>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="Q3" s="13" t="inlineStr">
         <is>
-          <t>Zero fitted parameters. All 41 parameters are empirically measured, physical constants, or derived coefficients. See parameter audit for details.</t>
+          <t>No per-pillar fitting: the parameter set is fixed before any validation pillar is evaluated. Within the set, β is anchored, α is frozen (void-motivated, not independently measured), τ is synchronised, and β_eos is fitted phenomenologically; remaining quantities are physical constants or derived coefficients. See parameter audit for details.</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="G4" s="16" t="inlineStr">
         <is>
-          <t>Consistent if one fixed parameter set, derived entirely from empirical or first-principles data and with no fitted parameters,
+          <t>Consistent if one parameter set, fixed in advance with no per-pillar fitting,
 reproduces all pillars within observational bands.</t>
         </is>
       </c>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Consistent if one fixed parameter set, derived entirely from empirical or first-principles data and with no fitted parameters,
+          <t>Consistent if one parameter set, fixed in advance with no per-pillar fitting,
 reproduces all pillars within observational bands.</t>
         </is>
       </c>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>Consistent if one fixed parameter set, derived entirely from empirical or first-principles data and with no fitted parameters,
+          <t>Consistent if one parameter set, fixed in advance with no per-pillar fitting,
 reproduces all pillars within observational bands.</t>
         </is>
       </c>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Consistent if one fixed parameter set, derived entirely from empirical or first-principles data and with no fitted parameters,
+          <t>Consistent if one parameter set, fixed in advance with no per-pillar fitting,
 reproduces all pillars within observational bands.</t>
         </is>
       </c>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G8" s="21" t="inlineStr">
         <is>
-          <t>Consistent if one fixed parameter set, derived entirely from empirical or first-principles data and with no fitted parameters,
+          <t>Consistent if one parameter set, fixed in advance with no per-pillar fitting,
 reproduces all pillars within observational bands.</t>
         </is>
       </c>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Observational anchor: consistent with cluster total baryon mass fractions at M_500 ~ 10^14 M_sun (range ~0.12-0.15); interpreted in the MTDF framework as an environmental coupling anchor. See MTDF_01 §5.1 note.</t>
+          <t>Fixed from cluster total baryon mass fractions at M_500 ~ 10^14 M_sun (range ~0.12-0.15; Giodini 2009, Gonzalez 2013); adopted post hoc as the environmental coupling value. This is the framework's largest open provenance weakness and an explicit falsification hook: an independent coupling measurement outside this range would falsify the assignment. See MTDF_01 §5.1 note.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Observational anchor under review: characteristic cluster core density at r_500 is consistent with X-ray hydrostatic mass profiles (Vikhlinin+2006 Chandra sample) and the REXCESS universal pressure profile (Arnaud+2010). The exact 6.4×10⁻²⁶ kg/m³ value requires re-derivation; see MTDF_01 §5.1 note.</t>
+          <t>External reference value under review: characteristic cluster core density at r_500 is consistent with X-ray hydrostatic mass profiles (Vikhlinin+2006 Chandra sample) and the REXCESS universal pressure profile (Arnaud+2010). The exact 6.4×10⁻²⁶ kg/m³ value requires re-derivation; see MTDF_01 §5.1 note.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -2667,7 +2667,7 @@
       <c r="A1" s="24" t="inlineStr">
         <is>
           <t>MTDF Fundamentals
-MTDF is governed by four independent inputs (α, β, τ, β_eos). E is defined from α, ρ_c, c and used throughout the equations for clarity. Each is independently measured or derived from universal physical principles, with full provenance. All other MTDF quantities ultimately reference these parameters. The field–baryon coupling (δ_bf), while functioning as a core correction term in MTDF’s stress-field dynamics, is empirically measured from cluster baryon fraction data. For provenance clarity it is placed under observational anchors, rather than listed here as a fundamental.</t>
+MTDF is governed by four independent inputs (α, β, τ, β_eos). E is defined from α, ρ_c, c and used throughout the equations for clarity. Provenance is mixed and documented per parameter: β is anchored to void statistics, α is frozen (void-motivated, not independently measured), τ is synchronised to the age of the universe, and β_eos is a fitted phenomenological exponent. All other MTDF quantities ultimately reference these parameters. The field–baryon coupling (δ_bf), while functioning as a core correction term in MTDF’s stress-field dynamics, is fixed from cluster baryon fraction data (adopted post hoc; see MTDF_01 §5.1). For provenance clarity it is placed under observational anchors, rather than listed here as a fundamental.</t>
         </is>
       </c>
       <c r="B1" s="97" t="n"/>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="D3" s="29" t="inlineStr">
         <is>
-          <t>Empirically measured from cosmic void dynamics; Represents ratio of stress-induced acceleration to gravitational acceleration; sets fundamental coupling strength between spacetime stress tensor and matter.</t>
+          <t>Frozen phenomenological coupling, motivated by cosmic void dynamics but not independently measured (the void pairing crosses volumes and methods; the SPARC inversion is mass-to-light sensitive; see MTDF_01 §5.0); represents the ratio of stress-induced to gravitational acceleration and sets the coupling strength between the spacetime stress tensor and matter.</t>
         </is>
       </c>
       <c r="E3" s="29" t="inlineStr">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Universal physics constant; Controls acceleration transition amplitude; connects MTDF to universal scaling laws of phase transitions.</t>
+          <t>Fitted phenomenological exponent (β_eos = 0.573 is an MTDF fit); controls the acceleration transition amplitude. Universal critical amplitudes (QCD, Landau-Ginzburg analogues) motivate the functional form, not the value.</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -8496,7 +8496,7 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;Foundation Classification&lt;/strong&gt;&lt;br&gt;Methodological basis for model predictions.&lt;br&gt;&lt;br&gt;&lt;em&gt;PUBLISHED:&lt;/em&gt; Model predictions sourced from peer-reviewed literature and established theoretical frameworks. Validation uses published parameter values and standard formulations.&lt;br&gt;&lt;br&gt;&lt;em&gt;EMPIRICAL:&lt;/em&gt; Model parameters empirically constrained from independent observations. No free parameters adjusted to fit validation tests.&lt;br&gt;&lt;br&gt;&lt;em&gt;THEORETICAL:&lt;/em&gt; Model requires theoretical extensions or hypothetical components beyond direct observational constraints.</t>
+          <t>&lt;strong&gt;Foundation Classification&lt;/strong&gt;&lt;br&gt;Methodological basis for model predictions.&lt;br&gt;&lt;br&gt;&lt;em&gt;PUBLISHED:&lt;/em&gt; Model predictions sourced from peer-reviewed literature and established theoretical frameworks. Validation uses published parameter values and standard formulations.&lt;br&gt;&lt;br&gt;&lt;em&gt;EMPIRICAL:&lt;/em&gt; Parameter set fixed in advance from a mix of anchored, frozen, synchronised, and fitted values (see parameter audit). No per-pillar free parameters adjusted to fit validation tests.&lt;br&gt;&lt;br&gt;&lt;em&gt;THEORETICAL:&lt;/em&gt; Model requires theoretical extensions or hypothetical components beyond direct observational constraints.</t>
         </is>
       </c>
       <c r="C38" s="15" t="inlineStr">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="L38" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;Foundation Classification&lt;/strong&gt;&lt;br&gt;Methodological basis for model predictions.&lt;br&gt;&lt;br&gt;&lt;em&gt;PUBLISHED:&lt;/em&gt; Model predictions sourced from peer-reviewed literature and established theoretical frameworks. Validation uses published parameter values and standard formulations.&lt;br&gt;&lt;br&gt;&lt;em&gt;EMPIRICAL:&lt;/em&gt; Model parameters empirically constrained from independent observations. No free parameters adjusted to fit validation tests.&lt;br&gt;&lt;br&gt;&lt;em&gt;THEORETICAL:&lt;/em&gt; Model requires theoretical extensions or hypothetical components beyond direct observational constraints.</t>
+          <t>&lt;strong&gt;Foundation Classification&lt;/strong&gt;&lt;br&gt;Methodological basis for model predictions.&lt;br&gt;&lt;br&gt;&lt;em&gt;PUBLISHED:&lt;/em&gt; Model predictions sourced from peer-reviewed literature and established theoretical frameworks. Validation uses published parameter values and standard formulations.&lt;br&gt;&lt;br&gt;&lt;em&gt;EMPIRICAL:&lt;/em&gt; Parameter set fixed in advance from a mix of anchored, frozen, synchronised, and fitted values (see parameter audit). No per-pillar free parameters adjusted to fit validation tests.&lt;br&gt;&lt;br&gt;&lt;em&gt;THEORETICAL:&lt;/em&gt; Model requires theoretical extensions or hypothetical components beyond direct observational constraints.</t>
         </is>
       </c>
       <c r="M38" s="16" t="inlineStr">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;Performance Classification&lt;/strong&gt;&lt;br&gt;Evidence assessment based on empirical tests.&lt;br&gt;&lt;br&gt;&lt;em&gt;✅ CONSISTENT:&lt;/em&gt; Achieves excellent fit (χ²/ν &lt; 0.1) across all tests using empirically constrained parameters only.&lt;br&gt;&lt;br&gt;&lt;em&gt;⚠️ REQUIRES_COMPONENTS:&lt;/em&gt; Requires hypothetical components not directly observed (dark matter, dark energy, modified gravity fields). May achieve good fits but invokes entities beyond current direct observational constraints.&lt;br&gt;&lt;br&gt;&lt;em&gt;❌ FAILED:&lt;/em&gt; Significant model-data tension (χ²/ν ≥ 2) or unable to provide predictions for critical observables.</t>
+          <t>&lt;strong&gt;Performance Classification&lt;/strong&gt;&lt;br&gt;Evidence assessment based on empirical tests.&lt;br&gt;&lt;br&gt;&lt;em&gt;✅ CONSISTENT:&lt;/em&gt; Within observational acceptance bands (χ²/ν &lt; 0.1 in the current scoring) across all strict tests with the pre-fixed parameter set; note that χ²/ν well below 1 can also reflect conservative uncertainties.&lt;br&gt;&lt;br&gt;&lt;em&gt;⚠️ REQUIRES_COMPONENTS:&lt;/em&gt; Requires hypothetical components not directly observed (dark matter, dark energy, modified gravity fields). May achieve good fits but invokes entities beyond current direct observational constraints.&lt;br&gt;&lt;br&gt;&lt;em&gt;❌ FAILED:&lt;/em&gt; Significant model-data tension (χ²/ν ≥ 2) or unable to provide predictions for critical observables.</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
@@ -8809,7 +8809,7 @@
       </c>
       <c r="L42" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;Performance Classification&lt;/strong&gt;&lt;br&gt;Evidence assessment based on empirical tests.&lt;br&gt;&lt;br&gt;&lt;em&gt;✅ CONSISTENT:&lt;/em&gt; Achieves excellent fit (χ²/ν &lt; 0.1) across all tests using empirically constrained parameters only.&lt;br&gt;&lt;br&gt;&lt;em&gt;⚠️ REQUIRES_COMPONENTS:&lt;/em&gt; Requires hypothetical components not directly observed (dark matter, dark energy, modified gravity fields). May achieve good fits but invokes entities beyond current direct observational constraints.&lt;br&gt;&lt;br&gt;&lt;em&gt;❌ FAILED:&lt;/em&gt; Significant model-data tension (χ²/ν ≥ 2) or unable to provide predictions for critical observables.</t>
+          <t>&lt;strong&gt;Performance Classification&lt;/strong&gt;&lt;br&gt;Evidence assessment based on empirical tests.&lt;br&gt;&lt;br&gt;&lt;em&gt;✅ CONSISTENT:&lt;/em&gt; Within observational acceptance bands (χ²/ν &lt; 0.1 in the current scoring) across all strict tests with the pre-fixed parameter set; note that χ²/ν well below 1 can also reflect conservative uncertainties.&lt;br&gt;&lt;br&gt;&lt;em&gt;⚠️ REQUIRES_COMPONENTS:&lt;/em&gt; Requires hypothetical components not directly observed (dark matter, dark energy, modified gravity fields). May achieve good fits but invokes entities beyond current direct observational constraints.&lt;br&gt;&lt;br&gt;&lt;em&gt;❌ FAILED:&lt;/em&gt; Significant model-data tension (χ²/ν ≥ 2) or unable to provide predictions for critical observables.</t>
         </is>
       </c>
       <c r="M42" s="16" t="inlineStr">
@@ -8923,7 +8923,7 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;Reduced Chi-Squared (χ²/ν)&lt;/strong&gt;&lt;br&gt;Normalized goodness-of-fit metric accounting for degrees of freedom.&lt;br&gt;&lt;br&gt;&lt;em&gt;Formula:&lt;/em&gt; χ²/ν = (Σz²) / (N − k)&lt;br&gt;where N = number of tests, k = free parameters&lt;br&gt;&lt;br&gt;&lt;em&gt;Quality benchmarks:&lt;/em&gt;&lt;br&gt;• χ²/ν &lt; 0.1: Excellent fit&lt;br&gt;• 0.1 ≤ χ²/ν &lt; 1: Strong agreement&lt;br&gt;• 1 ≤ χ²/ν &lt; 2: Acceptable fit&lt;br&gt;• χ²/ν ≥ 2: Model-data tension&lt;br&gt;&lt;br&gt;Statistical note: Well-fit models typically achieve χ²/ν ≈ 1. Values significantly below 1 indicate exceptional agreement or overfitting.</t>
+          <t>&lt;strong&gt;Reduced Chi-Squared (χ²/ν)&lt;/strong&gt;&lt;br&gt;Normalized goodness-of-fit metric accounting for degrees of freedom.&lt;br&gt;&lt;br&gt;&lt;em&gt;Formula:&lt;/em&gt; χ²/ν = (Σz²) / (N − k)&lt;br&gt;where N = number of tests, k = free parameters&lt;br&gt;&lt;br&gt;&lt;em&gt;Quality benchmarks:&lt;/em&gt;&lt;br&gt;• χ²/ν &lt; 0.1: Very small residuals (may reflect conservative uncertainties)&lt;br&gt;• 0.1 ≤ χ²/ν &lt; 1: Strong agreement&lt;br&gt;• 1 ≤ χ²/ν &lt; 2: Acceptable fit&lt;br&gt;• χ²/ν ≥ 2: Model-data tension&lt;br&gt;&lt;br&gt;Statistical note: Well-fit models typically achieve χ²/ν ≈ 1. Values significantly below 1 indicate exceptional agreement or overfitting.</t>
         </is>
       </c>
       <c r="C44" s="15" t="inlineStr">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="L44" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;Reduced Chi-Squared (χ²/ν)&lt;/strong&gt;&lt;br&gt;Normalized goodness-of-fit metric accounting for degrees of freedom.&lt;br&gt;&lt;br&gt;&lt;em&gt;Formula:&lt;/em&gt; χ²/ν = (Σz²) / (N − k)&lt;br&gt;where N = number of tests, k = free parameters&lt;br&gt;&lt;br&gt;&lt;em&gt;Quality benchmarks:&lt;/em&gt;&lt;br&gt;• χ²/ν &lt; 0.1: Excellent fit&lt;br&gt;• 0.1 ≤ χ²/ν &lt; 1: Strong agreement&lt;br&gt;• 1 ≤ χ²/ν &lt; 2: Acceptable fit&lt;br&gt;• χ²/ν ≥ 2: Model-data tension&lt;br&gt;&lt;br&gt;Statistical note: Well-fit models typically achieve χ²/ν ≈ 1. Values significantly below 1 indicate exceptional agreement or overfitting.</t>
+          <t>&lt;strong&gt;Reduced Chi-Squared (χ²/ν)&lt;/strong&gt;&lt;br&gt;Normalized goodness-of-fit metric accounting for degrees of freedom.&lt;br&gt;&lt;br&gt;&lt;em&gt;Formula:&lt;/em&gt; χ²/ν = (Σz²) / (N − k)&lt;br&gt;where N = number of tests, k = free parameters&lt;br&gt;&lt;br&gt;&lt;em&gt;Quality benchmarks:&lt;/em&gt;&lt;br&gt;• χ²/ν &lt; 0.1: Very small residuals (may reflect conservative uncertainties)&lt;br&gt;• 0.1 ≤ χ²/ν &lt; 1: Strong agreement&lt;br&gt;• 1 ≤ χ²/ν &lt; 2: Acceptable fit&lt;br&gt;• χ²/ν ≥ 2: Model-data tension&lt;br&gt;&lt;br&gt;Statistical note: Well-fit models typically achieve χ²/ν ≈ 1. Values significantly below 1 indicate exceptional agreement or overfitting.</t>
         </is>
       </c>
       <c r="M44" s="16" t="inlineStr">
@@ -9101,7 +9101,7 @@
       </c>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;Foundation Type&lt;/strong&gt;&lt;br&gt;Indicates the methodological basis for this model's predictions.&lt;br&gt;&lt;br&gt;PUBLISHED: Uses published parameter values from peer-reviewed literature&lt;br&gt;EMPIRICAL: Parameters constrained from independent observations&lt;br&gt;THEORETICAL: Requires theoretical extensions or hypothetical components&lt;br&gt;&lt;br&gt;Hover over specific foundation labels for detailed explanations.</t>
+          <t>&lt;strong&gt;Foundation Type&lt;/strong&gt;&lt;br&gt;Indicates the methodological basis for this model's predictions.&lt;br&gt;&lt;br&gt;PUBLISHED: Uses published parameter values from peer-reviewed literature&lt;br&gt;EMPIRICAL: Parameter set fixed in advance (anchored/frozen/synchronised/fitted mix; see parameter audit)&lt;br&gt;THEORETICAL: Requires theoretical extensions or hypothetical components&lt;br&gt;&lt;br&gt;Hover over specific foundation labels for detailed explanations.</t>
         </is>
       </c>
       <c r="C47" s="15" t="inlineStr">
@@ -9149,7 +9149,7 @@
       </c>
       <c r="L47" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;Foundation Type&lt;/strong&gt;&lt;br&gt;Indicates the methodological basis for this model's predictions.&lt;br&gt;&lt;br&gt;PUBLISHED: Uses published parameter values from peer-reviewed literature&lt;br&gt;EMPIRICAL: Parameters constrained from independent observations&lt;br&gt;THEORETICAL: Requires theoretical extensions or hypothetical components&lt;br&gt;&lt;br&gt;Hover over specific foundation labels for detailed explanations.</t>
+          <t>&lt;strong&gt;Foundation Type&lt;/strong&gt;&lt;br&gt;Indicates the methodological basis for this model's predictions.&lt;br&gt;&lt;br&gt;PUBLISHED: Uses published parameter values from peer-reviewed literature&lt;br&gt;EMPIRICAL: Parameter set fixed in advance (anchored/frozen/synchronised/fitted mix; see parameter audit)&lt;br&gt;THEORETICAL: Requires theoretical extensions or hypothetical components&lt;br&gt;&lt;br&gt;Hover over specific foundation labels for detailed explanations.</t>
         </is>
       </c>
       <c r="M47" s="16" t="inlineStr">
@@ -9506,7 +9506,7 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;Reduced χ²&lt;/strong&gt;&lt;br&gt;Goodness-of-fit metric for this model normalized by degrees of freedom.&lt;br&gt;&lt;br&gt;Lower values indicate better agreement with observations. Values &lt; 0.1 indicate excellent fit; values ≥ 2 indicate model-data tension requiring revision.</t>
+          <t>&lt;strong&gt;Reduced χ²&lt;/strong&gt;&lt;br&gt;Goodness-of-fit metric for this model normalized by degrees of freedom.&lt;br&gt;&lt;br&gt;Lower values indicate better agreement with observations. Values well below 1 indicate very small residuals (or conservative uncertainties); values ≥ 2 indicate model-data tension requiring revision.</t>
         </is>
       </c>
       <c r="C52" s="15" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="L52" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;Reduced χ²&lt;/strong&gt;&lt;br&gt;Goodness-of-fit metric for this model normalized by degrees of freedom.&lt;br&gt;&lt;br&gt;Lower values indicate better agreement with observations. Values &lt; 0.1 indicate excellent fit; values ≥ 2 indicate model-data tension requiring revision.</t>
+          <t>&lt;strong&gt;Reduced χ²&lt;/strong&gt;&lt;br&gt;Goodness-of-fit metric for this model normalized by degrees of freedom.&lt;br&gt;&lt;br&gt;Lower values indicate better agreement with observations. Values well below 1 indicate very small residuals (or conservative uncertainties); values ≥ 2 indicate model-data tension requiring revision.</t>
         </is>
       </c>
       <c r="M52" s="16" t="inlineStr">
@@ -11412,7 +11412,7 @@
       </c>
       <c r="B83" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;Foundation: MTDF (Tensor Dynamics)&lt;/strong&gt;&lt;br&gt;First-principles framework treating spacetime as an elastic medium.&lt;br&gt;&lt;br&gt;&lt;em&gt;Parameter constraints:&lt;/em&gt;&lt;br&gt;• α (stress-matter coupling): From SPARC galaxy rotation data&lt;br&gt;• β (coherence length): From void size quantization&lt;br&gt;• δ_bf (field-baryon coupling): From cluster observations&lt;br&gt;• E (elastic modulus): From β_eos and physical constraints&lt;br&gt;• β_eos (equation of state): From CMB polarization&lt;br&gt;&lt;br&gt;&lt;em&gt;Methodological distinction:&lt;/em&gt; All parameters empirically constrained from independent observations. No parameters adjusted to fit validation tests, preventing circular reasoning and ensuring genuine predictive power.</t>
+          <t>&lt;strong&gt;Foundation: MTDF (Tensor Dynamics)&lt;/strong&gt;&lt;br&gt;First-principles framework treating spacetime as an elastic medium.&lt;br&gt;&lt;br&gt;&lt;em&gt;Parameter provenance:&lt;/em&gt;&lt;br&gt;• α (stress-matter coupling): frozen void-motivated value, not independently measured (SPARC support is mass-to-light sensitive)&lt;br&gt;• β (coherence length): anchored to void statistics&lt;br&gt;• δ_bf (field-baryon coupling): fixed post hoc from cluster baryon fractions&lt;br&gt;• E (elastic modulus): derived from α&lt;br&gt;• β_eos (equation of state): fitted phenomenological exponent (CMB polarization analogue motivates the form, not the value)&lt;br&gt;&lt;br&gt;&lt;em&gt;Methodological distinction:&lt;/em&gt; The parameter set is fixed before validation and no quantity is adjusted per pillar; provenance is mixed (anchored, frozen, synchronised, fitted) and documented in the parameter audit.</t>
         </is>
       </c>
       <c r="C83" s="15" t="inlineStr">
@@ -11460,7 +11460,7 @@
       </c>
       <c r="L83" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;Foundation: MTDF (Tensor Dynamics)&lt;/strong&gt;&lt;br&gt;First-principles framework treating spacetime as an elastic medium.&lt;br&gt;&lt;br&gt;&lt;em&gt;Parameter constraints:&lt;/em&gt;&lt;br&gt;• α (stress-matter coupling): From SPARC galaxy rotation data&lt;br&gt;• β (coherence length): From void size quantization&lt;br&gt;• δ_bf (field-baryon coupling): From cluster observations&lt;br&gt;• E (elastic modulus): From β_eos and physical constraints&lt;br&gt;• β_eos (equation of state): From CMB polarization&lt;br&gt;&lt;br&gt;&lt;em&gt;Methodological distinction:&lt;/em&gt; All parameters empirically constrained from independent observations. No parameters adjusted to fit validation tests, preventing circular reasoning and ensuring genuine predictive power.</t>
+          <t>&lt;strong&gt;Foundation: MTDF (Tensor Dynamics)&lt;/strong&gt;&lt;br&gt;First-principles framework treating spacetime as an elastic medium.&lt;br&gt;&lt;br&gt;&lt;em&gt;Parameter provenance:&lt;/em&gt;&lt;br&gt;• α (stress-matter coupling): frozen void-motivated value, not independently measured (SPARC support is mass-to-light sensitive)&lt;br&gt;• β (coherence length): anchored to void statistics&lt;br&gt;• δ_bf (field-baryon coupling): fixed post hoc from cluster baryon fractions&lt;br&gt;• E (elastic modulus): derived from α&lt;br&gt;• β_eos (equation of state): fitted phenomenological exponent (CMB polarization analogue motivates the form, not the value)&lt;br&gt;&lt;br&gt;&lt;em&gt;Methodological distinction:&lt;/em&gt; The parameter set is fixed before validation and no quantity is adjusted per pillar; provenance is mixed (anchored, frozen, synchronised, fitted) and documented in the parameter audit.</t>
         </is>
       </c>
       <c r="N83" s="15" t="n">
@@ -12162,7 +12162,7 @@
       </c>
       <c r="L94" s="16" t="inlineStr">
         <is>
-          <t>&lt;strong&gt;χ²/ν: Reduced Chi-Squared&lt;/strong&gt;&lt;br&gt;Normalized goodness-of-fit: χ²/ν = (Total χ²) / (Degrees of freedom)&lt;br&gt;&lt;br&gt;&lt;em&gt;Statistical benchmarks:&lt;/em&gt;&lt;br&gt;• χ²/ν &lt; 0.1: Excellent fit&lt;br&gt;• 0.1 ≤ χ²/ν &lt; 1: Strong agreement&lt;br&gt;• 1 ≤ χ²/ν &lt; 2: Acceptable fit&lt;br&gt;• χ²/ν ≥ 2: Model-data tension</t>
+          <t>&lt;strong&gt;χ²/ν: Reduced Chi-Squared&lt;/strong&gt;&lt;br&gt;Normalized goodness-of-fit: χ²/ν = (Total χ²) / (Degrees of freedom)&lt;br&gt;&lt;br&gt;&lt;em&gt;Statistical benchmarks:&lt;/em&gt;&lt;br&gt;• χ²/ν &lt; 0.1: Very small residuals (may reflect conservative uncertainties)&lt;br&gt;• 0.1 ≤ χ²/ν &lt; 1: Strong agreement&lt;br&gt;• 1 ≤ χ²/ν &lt; 2: Acceptable fit&lt;br&gt;• χ²/ν ≥ 2: Model-data tension</t>
         </is>
       </c>
       <c r="N94" s="15" t="n">
@@ -13437,12 +13437,13 @@
           <t>&lt;strong&gt;MTDF (Mesche's Tensor Dynamics Framework)&lt;/strong&gt;&lt;br&gt;&lt;br&gt;
 Mesche's Tensor Dynamics Framework is an elastic spacetime field model that 
 replaces particle dark matter and dark energy with a continuous stress field. 
-The framework is defined by four fundamental parameters (α, β, τ, β_eos), with 
-all remaining quantities either derived from these or constrained by external 
-observations. No parameters are fitted to the validation pillars shown here.&lt;br&gt;&lt;br&gt;
+The framework is defined by four fundamental parameters with mixed, documented 
+provenance (one anchored β, one frozen void-motivated α, one synchronised τ, one 
+fitted β_eos); remaining quantities are derived or externally constrained. No 
+parameters are tuned per validation pillar.&lt;br&gt;&lt;br&gt;
 &lt;strong&gt;Key features in this dashboard:&lt;/strong&gt;&lt;br&gt;
 • No cold dark matter or cosmological constant; cosmic acceleration and galaxy dynamics arise from the elastic field response.&lt;br&gt;
-• Four fundamental parameters with all remaining quantities derived or externally constrained. No parameters are fitted to validation data.&lt;br&gt;
+• Four fundamental parameters (anchored β, frozen α, synchronised τ, fitted β_eos) with remaining quantities derived or externally constrained. No per-pillar parameter tuning.&lt;br&gt;
 • Provides a single, coherent description of late time expansion, structure growth, lensing and galactic dynamics across about 1700 degrees of freedom.</t>
         </is>
       </c>
@@ -14518,8 +14519,8 @@
         <is>
           <t>&lt;strong&gt;MTDF (EFE) - MTDF with Early Field Energy&lt;/strong&gt;&lt;br&gt;&lt;br&gt;
 This variant adds the analytically predicted early field energy bump around 
-matter-radiation equality. The EFE amplitude is fixed by the field theory, 
-with f_kick = λ_MTDF / 24 ≈ 0.33 percent, so there are no new free parameters 
+matter-radiation equality. The EFE amplitude is set by the field construction, 
+with f_kick = λ_MTDF / 24 ≈ 0.33 percent, (the 1/24 combines one exact and two heuristic geometric factors), so there are no new free parameters 
 beyond (α, β_eos, z_t).&lt;br&gt;&lt;br&gt;
 &lt;strong&gt;Key features in this dashboard:&lt;/strong&gt;&lt;br&gt;
 • Same late time elastic field as baseline MTDF; only early era physics differs through the predicted EFE bump.&lt;br&gt;
@@ -17622,6 +17623,11 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
     <row r="23" ht="15" customHeight="1">
       <c r="E23" s="5" t="n"/>
     </row>
@@ -17872,12 +17878,12 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>DOI: 10.1093/mnras/staa2073 (Bullet Cluster centroid offsets)</t>
+          <t>DOI: 10.1086/508162 (Clowe et al. 2006, Bullet Cluster 1E 0657-56 mass-gas offset / direct DM proof)</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Benchmark derived from updated centroid offset measurement; consistent across weak-lensing and X-ray studies</t>
+          <t>Benchmark derived from updated centroid offset measurement; consistent across weak-lensing and X-ray studies | [Audit 2026-06-10] source_doi was 10.1093/mnras/staa2073, which resolves to Mandal &amp; Nadkarni-Ghosh 2020 (spherical-collapse PDF, early dark energy) -- WRONG paper; replaced with Clowe et al. 2006 (10.1086/508162). NOTE: value 720 kpc = subcluster separation; observable label may need review vs mass-gas offset.</t>
         </is>
       </c>
       <c r="I5" s="44" t="n">
@@ -22189,6 +22195,15 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
     <row r="27" ht="15" customHeight="1">
       <c r="I27" s="57" t="n"/>
     </row>
@@ -28560,7 +28575,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Anchor: approx f_kick/3 (within FIRAS spectral-distortion bounds)</t>
+          <t>Theory-motivated: approx f_kick/3 (FIRAS spectral-distortion limits bound, but do not measure, this value)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -28585,7 +28600,7 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>[MTDF Foundations 2025] §3.9 Photon Coupling; Observational anchor, structurally related to f_kick/3 (angular averaging gives 1.10e-3, pipeline retains 1.02e-3); Fixsen et al. 1996, ApJ 473, 576</t>
+          <t>[MTDF Foundations 2025] §3.9 Photon Coupling; Theory-motivated value, structurally related to f_kick/3 (angular averaging gives 1.10e-3, pipeline retains 1.02e-3); FIRAS bounds but does not measure it; Fixsen et al. 1996, ApJ 473, 576</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">

</xml_diff>